<commit_message>
TICVAI: biometrics for children in the client email and Decisions Register (30 September meeting)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Decisions Register.xlsx
+++ b/ticvai/handoff/TICVAI - Decisions Register.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements closed" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Audit decisions'!$A$1:$G$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rev 3 prototype feedback'!$A$1:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Agreed operations'!$A$1:$E$575</definedName>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -930,32 +930,32 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Forecasting</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Weather data</t>
+          <t>Biometrics for children</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Do you approve a commercial weather data service as an input to attendance forecasting, and its monthly cost?</t>
+          <t>Adults may have face data stored with their consent. For guests under 18, should face capture (Face Pass, Face Tag) be excluded entirely, or allowed with a consent form signed by a parent or guardian? (Raised in the 30 September meeting.)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>A cost you approve</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Forecasts run on sales history, bookings on hand and the calendar (holidays, Ramadan) without weather until you approve.</t>
+          <t>Face capture is not offered to guests under 18 until you decide; with guardian consent, the guardian's signed consent is recorded against the child's ticket before capture.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Your commercial team</t>
+          <t>Your data protection counsel</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
@@ -966,32 +966,32 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Forecasting</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Design sign-off</t>
+          <t>Weather data</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Name one design reviewer who signs off each wireframe batch within 3 working days.</t>
+          <t>Do you approve a commercial weather data service as an input to attendance forecasting, and its monthly cost?</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>A name only you can give</t>
+          <t>A cost you approve</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Front-end screens are accepted only after that sign-off (decided 28 September).</t>
+          <t>Forecasts run on sales history, bookings on hand and the calendar (holidays, Ramadan) without weather until you approve.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Your product owner</t>
+          <t>Your commercial team</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
@@ -1007,27 +1007,27 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Payment sandboxes</t>
+          <t>Design sign-off</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Send Stripe and Network International sandbox credentials, and name the finance or payments owner, by a date we agree together.</t>
+          <t>Name one design reviewer who signs off each wireframe batch within 3 working days.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Accounts only you hold</t>
+          <t>A name only you can give</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Checkout's declined, unknown and reconcile paths cannot be tested without a sandbox.</t>
+          <t>Front-end screens are accepted only after that sign-off (decided 28 September).</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Your finance / payments owner</t>
+          <t>Your product owner</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -1038,32 +1038,32 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Accounts and people</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Cloud event broker</t>
+          <t>Payment sandboxes</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Which broker should carry the platform's events in the cloud: RabbitMQ or Kafka? We need your answer before 12 October (the second week of the first sprint), so that the first purchase can be proven end to end by 23 October. Why it matters: every sale reaches ticketing, the ledger and stock through this broker, so it must keep each order's events in sequence, set aside messages that fail, and run in the UAE. Our recommendation is RabbitMQ, ideally as a managed service in the Azure UAE North region if one is available there: it fits this workload, it is simpler to run, and venues that run on their own premises use RabbitMQ anyway. Kafka is the better choice only if you want to replay the history of events from the broker itself.</t>
+          <t>Send Stripe and Network International sandbox credentials, and name the finance or payments owner, by a date we agree together.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>A platform and running cost you choose</t>
+          <t>Accounts only you hold</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Everything is built behind one interface and tested on RabbitMQ, so either answer works; only the cloud setup waits for your choice.</t>
+          <t>Checkout's declined, unknown and reconcile paths cannot be tested without a sandbox.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Your IT / infrastructure owner</t>
+          <t>Your finance / payments owner</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr"/>
@@ -1074,32 +1074,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>POS terminal</t>
+          <t>Cloud event broker</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Which POS terminal will the cashiers use: make, model and operating system (Windows, Android or iPad)? Your hardware list names the receipt printer, cash drawer, customer display and scanner, but not the terminal.</t>
+          <t>Which broker should carry the platform's events in the cloud: RabbitMQ or Kafka? We need your answer before 12 October (the second week of the first sprint), so that the first purchase can be proven end to end by 23 October. Why it matters: every sale reaches ticketing, the ledger and stock through this broker, so it must keep each order's events in sequence, set aside messages that fail, and run in the UAE. Our recommendation is RabbitMQ, ideally as a managed service in the Azure UAE North region if one is available there: it fits this workload, it is simpler to run, and venues that run on their own premises use RabbitMQ anyway. Kafka is the better choice only if you want to replay the history of events from the broker itself.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>A platform and running cost you choose</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>The POS is built as an app that works offline and drives the printer, drawer and display through standard drivers. We assume a Windows touch terminal (the HP cash drawer, display and scanner on your list suggest an HP POS system); the operating system decides how those devices are driven, so we need it before the first sprint ends.</t>
+          <t>Everything is built behind one interface and tested on RabbitMQ, so either answer works; only the cloud setup waits for your choice.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your IT / infrastructure owner</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Kitchen display</t>
+          <t>POS terminal</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Which kitchen display screens and kitchen printers will the kitchens use? Your hardware list says "decide later", and the kitchen display is in the first release.</t>
+          <t>Which POS terminal will the cashiers use: make, model and operating system (Windows, Android or iPad)? Your hardware list names the receipt printer, cash drawer, customer display and scanner, but not the terminal.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>The kitchen display is built as a browser screen that runs on any wall-mounted touch screen or tablet, with kitchen tickets also printable on an Epson-compatible printer.</t>
+          <t>The POS is built as an app that works offline and drives the printer, drawer and display through standard drivers. We assume a Windows touch terminal (the HP cash drawer, display and scanner on your list suggest an HP POS system); the operating system decides how those devices are driven, so we need it before the first sprint ends.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Your F&amp;B / operations team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
@@ -1151,27 +1151,27 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Card payment terminals</t>
+          <t>Kitchen display</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Which card payment terminals will the POS and the kiosks use, and from which provider (Stripe Terminal, Network International, or another)? They are not on your hardware list.</t>
+          <t>Which kitchen display screens and kitchen printers will the kitchens use? Your hardware list says "decide later", and the kitchen display is in the first release.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>A device and a merchant contract only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Card payments at the POS go through the payment provider's terminal, paired to one POS; the POS never sees a card number. Until you name the terminal, testing uses the provider's simulator.</t>
+          <t>The kitchen display is built as a browser screen that runs on any wall-mounted touch screen or tablet, with kitchen tickets also printable on an Epson-compatible printer.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Your finance / payments owner</t>
+          <t>Your F&amp;B / operations team</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
@@ -1187,27 +1187,27 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>NFC and RFID media</t>
+          <t>Card payment terminals</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Which NFC readers (your list says "China") and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
+          <t>Which card payment terminals will the POS and the kiosks use, and from which provider (Stripe Terminal, Network International, or another)? They are not on your hardware list.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>A device and a merchant contract only you hold</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Wristbands and cards are read by their unique id and a secured application on the chip; nothing of value is stored on the chip itself. The exact chip type sets how the encoder is driven.</t>
+          <t>Card payments at the POS go through the payment provider's terminal, paired to one POS; the POS never sees a card number. Until you name the terminal, testing uses the provider's simulator.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your finance / payments owner</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr"/>
@@ -1223,12 +1223,12 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Staff and flying POS devices</t>
+          <t>NFC and RFID media</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Will the staff app and the flying (handheld) POS run on the Chainway C66 handhelds on your list, or on other phones or tablets?</t>
+          <t>Which NFC readers (your list says "China") and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1238,12 +1238,12 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Both are built as one Android app for the Chainway C66, which also scans and prints over Bluetooth to the Zebra printer.</t>
+          <t>Wristbands and cards are read by their unique id and a secured application on the chip; nothing of value is stored on the chip itself. The exact chip type sets how the encoder is driven.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Your operations team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr"/>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Devices in the requirements but not on your hardware list</t>
+          <t>Staff and flying POS devices</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
+          <t>Will the staff app and the flying (handheld) POS run on the Chainway C66 handhelds on your list, or on other phones or tablets?</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
+          <t>Both are built as one Android app for the Chainway C66, which also scans and prints over Bluetooth to the Zebra printer.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your operations team</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr"/>
@@ -1290,32 +1290,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Messaging providers</t>
+          <t>Devices in the requirements but not on your hardware list</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
+          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
+          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr"/>
@@ -1331,27 +1331,27 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Accounting system</t>
+          <t>Messaging providers</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
+          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>A system and a format only you hold</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
+          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Your finance team</t>
+          <t>Your IT / marketing team</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr"/>
@@ -1367,27 +1367,27 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass</t>
+          <t>Accounting system</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
+          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A system and a format only you hold</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
+          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Your IT team</t>
+          <t>Your finance team</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr"/>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>App stores and digital wallets</t>
+          <t>UAE Pass</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
+          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1418,12 +1418,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
+          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Your IT team</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr"/>
@@ -1434,32 +1434,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Tourism authority reporting</t>
+          <t>App stores and digital wallets</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
+          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
+          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Your compliance / finance team</t>
+          <t>Your IT / marketing team</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr"/>
@@ -1470,32 +1470,32 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Government</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Named third-party services</t>
+          <t>Tourism authority reporting</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
+          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Your commercial / operations team</t>
+          <t>Your compliance / finance team</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr"/>
@@ -1506,30 +1506,34 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Guardian consent for a minor's Face Pass (sent before)</t>
+          <t>Named third-party services</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
+          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr"/>
+          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Your commercial / operations team</t>
+        </is>
+      </c>
       <c r="H24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1543,12 +1547,12 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>The age of a minor (sent before)</t>
+          <t>Guardian consent for a minor's Face Pass (sent before)</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Below what age is a guest a minor?</t>
+          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1558,7 +1562,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
+          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr"/>
@@ -1575,12 +1579,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Guest document retention (sent before)</t>
+          <t>The age of a minor (sent before)</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>How long is each kind of guest document kept?</t>
+          <t>Below what age is a guest a minor?</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1590,7 +1594,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
+          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr"/>
@@ -1602,27 +1606,27 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Refunds</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Cancelled event after a resale (sent before)</t>
+          <t>Guest document retention (sent before)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
+          <t>How long is each kind of guest document kept?</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Money your customers pay or get back</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr"/>
@@ -1634,27 +1638,27 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Refunds</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Facial-reader vendor (sent before)</t>
+          <t>Cancelled event after a resale (sent before)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Money your customers pay or get back</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
+          <t>Kept open in the specification; the rest is built.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
@@ -1666,17 +1670,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Approved libraries (sent before)</t>
+          <t>Facial-reader vendor (sent before)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1686,7 +1690,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
+          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
@@ -1698,27 +1702,27 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Accounts and people</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Price tests on live customers (sent before)</t>
+          <t>Approved libraries (sent before)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr"/>
@@ -1735,12 +1739,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Cooling-off after auto-renewal (sent before)</t>
+          <t>Price tests on live customers (sent before)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1756,8 +1760,40 @@
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="7" t="inlineStr"/>
     </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Cooling-off after auto-renewal (sent before)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H31"/>
+  <autoFilter ref="A1:H32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TICVAI: 30 September changes, pre-release state (refresh of 30 Sep evening; final checks not yet run)
Planner multi-venue + retail and ride video without loader (MoM 4.7, 4.8); ADR-0069 in-park 3D navigation;
AI billing deferred (AI-D20); children's biometrics and 3D venue model questions; infra answers applied
(Azure Managed Redis, cost sheet, Terraform network, ADR-0049/0057/0032); stable ticket keys
(check-key-stability); Claude Design run sheets. Checks and the r1 tag follow on this branch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Decisions Register.xlsx
+++ b/ticvai/handoff/TICVAI - Decisions Register.xlsx
@@ -17,12 +17,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements closed" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Audit decisions'!$A$1:$G$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rev 3 prototype feedback'!$A$1:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Agreed operations'!$A$1:$E$575</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Operations added'!$A$1:$D$207</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'AI decisions'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'AI decisions'!$A$1:$C$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Requirements closed'!$A$1:$F$531</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Which NFC readers (your list says "China") and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
+          <t>Which NFC readers (your list says "China", still open) and RFID readers (Kaptur, still open), and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1542,30 +1542,34 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Venue data</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Guardian consent for a minor's Face Pass (sent before)</t>
+          <t>3D venue model for in-park navigation</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
+          <t>In-park 3D navigation is built into the guest app, as agreed on 30 September, and needs two files for each venue: a 3D model of the venue (a GLB file) and a pathway and location file (the walkable paths, and where each ride, outlet, shop and facility is, linked to its catalogue item), with two or more surveyed GPS points so the model lines up with the guest's position. Will you supply these for each venue, or commission a 3D vendor to produce them, and by when? We will send the file specification.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>Your venue's own asset, or a cost you approve</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr"/>
+          <t>In-park navigation runs on the 2D park map, with the same routes and live GPS, until a venue's model is supplied; the 3D view switches on per venue when its files pass the platform's checks.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Your operations / venue team</t>
+        </is>
+      </c>
       <c r="H25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1579,12 +1583,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>The age of a minor (sent before)</t>
+          <t>Guardian consent for a minor's Face Pass (sent before)</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Below what age is a guest a minor?</t>
+          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1594,7 +1598,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
+          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr"/>
@@ -1611,12 +1615,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Guest document retention (sent before)</t>
+          <t>The age of a minor (sent before)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>How long is each kind of guest document kept?</t>
+          <t>Below what age is a guest a minor?</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1626,7 +1630,7 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
+          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr"/>
@@ -1638,27 +1642,27 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Refunds</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Cancelled event after a resale (sent before)</t>
+          <t>Guest document retention (sent before)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
+          <t>How long is each kind of guest document kept?</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Money your customers pay or get back</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
@@ -1670,27 +1674,27 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Refunds</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Facial-reader vendor (sent before)</t>
+          <t>Cancelled event after a resale (sent before)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Money your customers pay or get back</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
+          <t>Kept open in the specification; the rest is built.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
@@ -1702,17 +1706,17 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Approved libraries (sent before)</t>
+          <t>Facial-reader vendor (sent before)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1722,7 +1726,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
+          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr"/>
@@ -1734,27 +1738,27 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Accounts and people</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Price tests on live customers (sent before)</t>
+          <t>Approved libraries (sent before)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr"/>
@@ -1771,12 +1775,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Cooling-off after auto-renewal (sent before)</t>
+          <t>Price tests on live customers (sent before)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1792,8 +1796,40 @@
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="7" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Cooling-off after auto-renewal (sent before)</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H32"/>
+  <autoFilter ref="A1:H33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26176,7 +26212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -26524,8 +26560,25 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>AI-D20</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>AI model billing when a client picks its own provider or model</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>DEFERRED, not decided: to the dedicated AI workshop (client meeting 30 September, MoM 4.1; Allam). Position stated on the call, for the workshop to confirm: the AI agents behave the same whichever model a client selects, with only minor performance variation; we propose a recommended model per function; any extra cost of a provider or model the client chooses (for example ChatGPT) is borne by the client. Until the workshop, AI-D02 (managed Azure OpenAI, re-billed per token) stands as the default</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C20"/>
+  <autoFilter ref="A1:C21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TICVAI: 4 client questions from ADR-0060/0062/0063 in the Decisions Register (36)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Decisions Register.xlsx
+++ b/ticvai/handoff/TICVAI - Decisions Register.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements closed" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Audit decisions'!$A$1:$G$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rev 3 prototype feedback'!$A$1:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Agreed operations'!$A$1:$E$575</definedName>
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Prepared by Softlabs · 30 September 2026 · generated from the specification package</t>
+          <t>Prepared by Softlabs · 1 October 2026 · generated from the specification package</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -822,32 +822,32 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Tax documents</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Face capture on a notice</t>
+          <t>B2C e-invoices</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>May a guest be enrolled for Face Tag on a displayed notice alone, with no action from them, under the UAE PDPL?</t>
+          <t>Are e-invoices to consumers (B2C) outside the first phase of the UAE mandate for you, so only B2B invoices go through the provider at launch? (ADR-0062)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>The guest must actively agree on screen before capture. The notice-only option is not offered.</t>
+          <t>B2B invoices go through the provider; B2C receipts are issued by the platform and can be switched to the provider per venue when your mandate covers them.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Your data protection counsel</t>
+          <t>Your finance team</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr"/>
@@ -858,32 +858,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Identity verification provider</t>
+          <t>What 99.99% covers</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Do you use an external identity-verification provider for guest ID documents, and if so which one?</t>
+          <t>Which services does the 99.99% availability commitment cover: the whole platform, or the guest purchase and admission path only? And do you accept a separate target per tier (for example 99.99% for purchase and admission, 99.9% for back office and reporting)? (ADR-0060)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Guest ID documents are reviewed by your staff.</t>
+          <t>Purchase and admission are designed to 99.99%; back office, reporting and AI to 99.9%.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Your operations team</t>
+          <t>Your IT owner</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr"/>
@@ -894,17 +894,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Biometric retention by law</t>
+          <t>Zone-redundant hosting cost</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>What minimum or maximum retention does the law require for Face Pass, Face Tag and failed or abandoned captures, in each region you operate? (Asked before; restated with what we built.)</t>
+          <t>99.99% needs zone-redundant hosting in UAE North: about USD 8,050 a month against about USD 4,530 without it. Do you accept that cost for production? (ADR-0060, the Azure cost sheet)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Face Tag deleted once the ticket is fully used; Face Pass retention set by each venue. The legal limit you confirm becomes a floor no venue setting can go below.</t>
+          <t>Production is costed zone-redundant; pre-production is not.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Your data protection counsel</t>
+          <t>Your budget owner</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr"/>
@@ -935,12 +935,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Biometrics for children</t>
+          <t>Where face templates are stored</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Adults may have face data stored with their consent. For guests under 18, should face capture (Face Pass, Face Tag) be excluded entirely, or allowed with a consent form signed by a parent or guardian? (Raised in the 30 September meeting.)</t>
+          <t>Where may face templates be stored: only inside the facial-reader vendor's system at the venue, or also in the platform in UAE North (encrypted, with a key per tenant)? (ADR-0063)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -950,12 +950,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Face capture is not offered to guests under 18 until you decide; with guardian consent, the guardian's signed consent is recorded against the child's ticket before capture.</t>
+          <t>Templates stay with the reader vendor; the platform keeps only a reference and the guest's consent.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Your data protection counsel</t>
+          <t>Your data protection officer</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
@@ -966,32 +966,32 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Forecasting</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Weather data</t>
+          <t>Face capture on a notice</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Do you approve a commercial weather data service as an input to attendance forecasting, and its monthly cost?</t>
+          <t>May a guest be enrolled for Face Tag on a displayed notice alone, with no action from them, under the UAE PDPL?</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>A cost you approve</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Forecasts run on sales history, bookings on hand and the calendar (holidays, Ramadan) without weather until you approve.</t>
+          <t>The guest must actively agree on screen before capture. The notice-only option is not offered.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Your commercial team</t>
+          <t>Your data protection counsel</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
@@ -1002,32 +1002,32 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Design sign-off</t>
+          <t>Identity verification provider</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Name one design reviewer who signs off each wireframe batch within 3 working days.</t>
+          <t>Do you use an external identity-verification provider for guest ID documents, and if so which one?</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>A name only you can give</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Front-end screens are accepted only after that sign-off (decided 28 September).</t>
+          <t>Guest ID documents are reviewed by your staff.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Your product owner</t>
+          <t>Your operations team</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -1038,32 +1038,32 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Payment sandboxes</t>
+          <t>Biometric retention by law</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Send Stripe and Network International sandbox credentials, and name the finance or payments owner, by a date we agree together.</t>
+          <t>What minimum or maximum retention does the law require for Face Pass, Face Tag and failed or abandoned captures, in each region you operate? (Asked before; restated with what we built.)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Accounts only you hold</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Checkout's declined, unknown and reconcile paths cannot be tested without a sandbox.</t>
+          <t>Face Tag deleted once the ticket is fully used; Face Pass retention set by each venue. The legal limit you confirm becomes a floor no venue setting can go below.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Your finance / payments owner</t>
+          <t>Your data protection counsel</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr"/>
@@ -1074,32 +1074,32 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Cloud event broker</t>
+          <t>Biometrics for children</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Which broker should carry the platform's events in the cloud: RabbitMQ or Kafka? We need your answer before 12 October (the second week of the first sprint), so that the first purchase can be proven end to end by 23 October. Why it matters: every sale reaches ticketing, the ledger and stock through this broker, so it must keep each order's events in sequence, set aside messages that fail, and run in the UAE. Our recommendation is RabbitMQ, ideally as a managed service in the Azure UAE North region if one is available there: it fits this workload, it is simpler to run, and venues that run on their own premises use RabbitMQ anyway. Kafka is the better choice only if you want to replay the history of events from the broker itself.</t>
+          <t>Adults may have face data stored with their consent. For guests under 18, should face capture (Face Pass, Face Tag) be excluded entirely, or allowed with a consent form signed by a parent or guardian? (Raised in the 30 September meeting.)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>A platform and running cost you choose</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Everything is built behind one interface and tested on RabbitMQ, so either answer works; only the cloud setup waits for your choice.</t>
+          <t>Face capture is not offered to guests under 18 until you decide; with guardian consent, the guardian's signed consent is recorded against the child's ticket before capture.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Your IT / infrastructure owner</t>
+          <t>Your data protection counsel</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -1110,32 +1110,32 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Forecasting</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>POS terminal</t>
+          <t>Weather data</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Which POS terminal will the cashiers use: make, model and operating system (Windows, Android or iPad)? Your hardware list names the receipt printer, cash drawer, customer display and scanner, but not the terminal.</t>
+          <t>Do you approve a commercial weather data service as an input to attendance forecasting, and its monthly cost?</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>A cost you approve</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>The POS is built as an app that works offline and drives the printer, drawer and display through standard drivers. We assume a Windows touch terminal (the HP cash drawer, display and scanner on your list suggest an HP POS system); the operating system decides how those devices are driven, so we need it before the first sprint ends.</t>
+          <t>Forecasts run on sales history, bookings on hand and the calendar (holidays, Ramadan) without weather until you approve.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your commercial team</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
@@ -1146,32 +1146,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Accounts and people</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Kitchen display</t>
+          <t>Design sign-off</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Which kitchen display screens and kitchen printers will the kitchens use? Your hardware list says "decide later", and the kitchen display is in the first release.</t>
+          <t>Name one design reviewer who signs off each wireframe batch within 3 working days.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>A name only you can give</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>The kitchen display is built as a browser screen that runs on any wall-mounted touch screen or tablet, with kitchen tickets also printable on an Epson-compatible printer.</t>
+          <t>Front-end screens are accepted only after that sign-off (decided 28 September).</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Your F&amp;B / operations team</t>
+          <t>Your product owner</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
@@ -1182,27 +1182,27 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Accounts and people</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Card payment terminals</t>
+          <t>Payment sandboxes</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Which card payment terminals will the POS and the kiosks use, and from which provider (Stripe Terminal, Network International, or another)? They are not on your hardware list.</t>
+          <t>Send Stripe and Network International sandbox credentials, and name the finance or payments owner, by a date we agree together.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>A device and a merchant contract only you hold</t>
+          <t>Accounts only you hold</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Card payments at the POS go through the payment provider's terminal, paired to one POS; the POS never sees a card number. Until you name the terminal, testing uses the provider's simulator.</t>
+          <t>Checkout's declined, unknown and reconcile paths cannot be tested without a sandbox.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1218,32 +1218,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>NFC and RFID media</t>
+          <t>Cloud event broker</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Which NFC readers (your list says "China", still open) and RFID readers (Kaptur, still open), and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
+          <t>Which broker should carry the platform's events in the cloud: RabbitMQ or Kafka? We need your answer before 12 October (the second week of the first sprint), so that the first purchase can be proven end to end by 23 October. Why it matters: every sale reaches ticketing, the ledger and stock through this broker, so it must keep each order's events in sequence, set aside messages that fail, and run in the UAE. Our recommendation is RabbitMQ, ideally as a managed service in the Azure UAE North region if one is available there: it fits this workload, it is simpler to run, and venues that run on their own premises use RabbitMQ anyway. Kafka is the better choice only if you want to replay the history of events from the broker itself.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>A platform and running cost you choose</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Wristbands and cards are read by their unique id and a secured application on the chip; nothing of value is stored on the chip itself. The exact chip type sets how the encoder is driven.</t>
+          <t>Everything is built behind one interface and tested on RabbitMQ, so either answer works; only the cloud setup waits for your choice.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your IT / infrastructure owner</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr"/>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Staff and flying POS devices</t>
+          <t>POS terminal</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Will the staff app and the flying (handheld) POS run on the Chainway C66 handhelds on your list, or on other phones or tablets?</t>
+          <t>Which POS terminal will the cashiers use: make, model and operating system (Windows, Android or iPad)? Your hardware list names the receipt printer, cash drawer, customer display and scanner, but not the terminal.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1274,12 +1274,12 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Both are built as one Android app for the Chainway C66, which also scans and prints over Bluetooth to the Zebra printer.</t>
+          <t>The POS is built as an app that works offline and drives the printer, drawer and display through standard drivers. We assume a Windows touch terminal (the HP cash drawer, display and scanner on your list suggest an HP POS system); the operating system decides how those devices are driven, so we need it before the first sprint ends.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Your operations team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr"/>
@@ -1295,12 +1295,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Devices in the requirements but not on your hardware list</t>
+          <t>Kitchen display</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
+          <t>Which kitchen display screens and kitchen printers will the kitchens use? Your hardware list says "decide later", and the kitchen display is in the first release.</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1310,12 +1310,12 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
+          <t>The kitchen display is built as a browser screen that runs on any wall-mounted touch screen or tablet, with kitchen tickets also printable on an Epson-compatible printer.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your F&amp;B / operations team</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr"/>
@@ -1326,32 +1326,32 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Messaging providers</t>
+          <t>Card payment terminals</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
+          <t>Which card payment terminals will the POS and the kiosks use, and from which provider (Stripe Terminal, Network International, or another)? They are not on your hardware list.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device and a merchant contract only you hold</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
+          <t>Card payments at the POS go through the payment provider's terminal, paired to one POS; the POS never sees a card number. Until you name the terminal, testing uses the provider's simulator.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Your finance / payments owner</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr"/>
@@ -1362,32 +1362,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Accounting system</t>
+          <t>NFC and RFID media</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
+          <t>Which NFC readers (your list says "China", still open) and RFID readers (Kaptur, still open), and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>A system and a format only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
+          <t>Wristbands and cards are read by their unique id and a secured application on the chip; nothing of value is stored on the chip itself. The exact chip type sets how the encoder is driven.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Your finance team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr"/>
@@ -1398,32 +1398,32 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass</t>
+          <t>Staff and flying POS devices</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
+          <t>Will the staff app and the flying (handheld) POS run on the Chainway C66 handhelds on your list, or on other phones or tablets?</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
+          <t>Both are built as one Android app for the Chainway C66, which also scans and prints over Bluetooth to the Zebra printer.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Your IT team</t>
+          <t>Your operations team</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr"/>
@@ -1434,32 +1434,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>App stores and digital wallets</t>
+          <t>Devices in the requirements but not on your hardware list</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
+          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
+          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr"/>
@@ -1470,32 +1470,32 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Tourism authority reporting</t>
+          <t>Messaging providers</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
+          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
+          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Your compliance / finance team</t>
+          <t>Your IT / marketing team</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr"/>
@@ -1511,27 +1511,27 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Named third-party services</t>
+          <t>Accounting system</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
+          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>A system and a format only you hold</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Your commercial / operations team</t>
+          <t>Your finance team</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr"/>
@@ -1542,32 +1542,32 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Venue data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>3D venue model for in-park navigation</t>
+          <t>UAE Pass</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>In-park 3D navigation is built into the guest app, as agreed on 30 September, and needs two files for each venue: a 3D model of the venue (a GLB file) and a pathway and location file (the walkable paths, and where each ride, outlet, shop and facility is, linked to its catalogue item), with two or more surveyed GPS points so the model lines up with the guest's position. Will you supply these for each venue, or commission a 3D vendor to produce them, and by when? We will send the file specification.</t>
+          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Your venue's own asset, or a cost you approve</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>In-park navigation runs on the 2D park map, with the same routes and live GPS, until a venue's model is supplied; the 3D view switches on per venue when its files pass the platform's checks.</t>
+          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Your operations / venue team</t>
+          <t>Your IT team</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr"/>
@@ -1578,30 +1578,34 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Guardian consent for a minor's Face Pass (sent before)</t>
+          <t>App stores and digital wallets</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
+          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr"/>
+          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Your IT / marketing team</t>
+        </is>
+      </c>
       <c r="H26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1610,17 +1614,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Government</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>The age of a minor (sent before)</t>
+          <t>Tourism authority reporting</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Below what age is a guest a minor?</t>
+          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1630,10 +1634,14 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr"/>
+          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Your compliance / finance team</t>
+        </is>
+      </c>
       <c r="H27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1642,30 +1650,34 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Guest document retention (sent before)</t>
+          <t>Named third-party services</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>How long is each kind of guest document kept?</t>
+          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr"/>
+          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Your commercial / operations team</t>
+        </is>
+      </c>
       <c r="H28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1674,30 +1686,34 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Refunds</t>
+          <t>Venue data</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Cancelled event after a resale (sent before)</t>
+          <t>3D venue model for in-park navigation</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
+          <t>In-park 3D navigation is built into the guest app, as agreed on 30 September, and needs two files for each venue: a 3D model of the venue (a GLB file) and a pathway and location file (the walkable paths, and where each ride, outlet, shop and facility is, linked to its catalogue item), with two or more surveyed GPS points so the model lines up with the guest's position. Will you supply these for each venue, or commission a 3D vendor to produce them, and by when? We will send the file specification.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Money your customers pay or get back</t>
+          <t>Your venue's own asset, or a cost you approve</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr"/>
+          <t>In-park navigation runs on the 2D park map, with the same routes and live GPS, until a venue's model is supplied; the 3D view switches on per venue when its files pass the platform's checks.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Your operations / venue team</t>
+        </is>
+      </c>
       <c r="H29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1706,27 +1722,27 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Facial-reader vendor (sent before)</t>
+          <t>Guardian consent for a minor's Face Pass (sent before)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
+          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr"/>
@@ -1738,27 +1754,27 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Approved libraries (sent before)</t>
+          <t>The age of a minor (sent before)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+          <t>Below what age is a guest a minor?</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
+          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr"/>
@@ -1770,17 +1786,17 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Price tests on live customers (sent before)</t>
+          <t>Guest document retention (sent before)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+          <t>How long is each kind of guest document kept?</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1790,7 +1806,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr"/>
@@ -1802,22 +1818,22 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Refunds</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Cooling-off after auto-renewal (sent before)</t>
+          <t>Cancelled event after a resale (sent before)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>Money your customers pay or get back</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -1828,8 +1844,136 @@
       <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="7" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Suppliers</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Facial-reader vendor (sent before)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>A name, account or vendor only you hold</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Accounts and people</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Approved libraries (sent before)</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>A name, account or vendor only you hold</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr"/>
+      <c r="H35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Price tests on live customers (sent before)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Cooling-off after auto-renewal (sent before)</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H33"/>
+  <autoFilter ref="A1:H37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TICVAI: 6 client questions from the 30 September guest feedback (group booking, swim ability, popular routes); register at 42
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Decisions Register.xlsx
+++ b/ticvai/handoff/TICVAI - Decisions Register.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements closed" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Audit decisions'!$A$1:$G$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rev 3 prototype feedback'!$A$1:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Agreed operations'!$A$1:$E$575</definedName>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -822,32 +822,32 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tax documents</t>
+          <t>Group booking</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>B2C e-invoices</t>
+          <t>Supervisors</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Are e-invoices to consumers (B2C) outside the first phase of the UAE mandate for you, so only B2B invoices go through the provider at launch? (ADR-0062)</t>
+          <t>Your build lists supervisors separately and free. How many supervisors come free per group (per N guests), and is that per group ticket?</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>B2B invoices go through the provider; B2C receipts are issued by the platform and can be switched to the provider per venue when your mandate covers them.</t>
+          <t>Supervisors are a separate, free guest type, up to 1 per 10 guests, counted on the group request.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Your finance team</t>
+          <t>Your commercial team</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr"/>
@@ -858,32 +858,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Group booking</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>What 99.99% covers</t>
+          <t>Group types</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Which services does the 99.99% availability commitment cover: the whole platform, or the guest purchase and admission path only? And do you accept a separate target per tier (for example 99.99% for purchase and admission, 99.9% for back office and reporting)? (ADR-0060)</t>
+          <t>Your build shows School, Corporate, Tour operator and Community groups; the platform has general, school, corporate and party. Do tour operator and community become their own types, or map to general?</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Purchase and admission are designed to 99.99%; back office, reporting and AI to 99.9%.</t>
+          <t>Tour operator and community are added as their own group types.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Your IT owner</t>
+          <t>Your commercial team</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr"/>
@@ -894,32 +894,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Group booking</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Zone-redundant hosting cost</t>
+          <t>Minimum group size</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>99.99% needs zone-redundant hosting in UAE North: about USD 8,050 a month against about USD 4,530 without it. Do you accept that cost for production? (ADR-0060, the Azure cost sheet)</t>
+          <t>Each group ticket card shows a minimum group size. Is the minimum set per group ticket (product), and what are the values?</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Production is costed zone-redundant; pre-production is not.</t>
+          <t>Each group ticket carries its own minimum, default 10.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Your budget owner</t>
+          <t>Your commercial team</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr"/>
@@ -930,32 +930,32 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Group booking</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Where face templates are stored</t>
+          <t>Water-park groups by session</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Where may face templates be stored: only inside the facial-reader vendor's system at the venue, or also in the platform in UAE North (encrypted, with a key per tenant)? (ADR-0063)</t>
+          <t>Your build has a water-park group pick a session first; group requests today take a date only. Are water-park groups booked into a session?</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Templates stay with the reader vendor; the platform keeps only a reference and the guest's consent.</t>
+          <t>Group requests take a date and, for session-based products, a session.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Your data protection officer</t>
+          <t>Your operations team</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
@@ -966,17 +966,17 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Guest safety</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Face capture on a notice</t>
+          <t>Swim ability</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>May a guest be enrolled for Face Tag on a displayed notice alone, with no action from them, under the UAE PDPL?</t>
+          <t>The swim answer now changes what is offered: all swimmers see everything, some get a 'swim vests needed' counter, and none see a cheaper splash-and-river pass without slides. Is the vest an add-on product, and is the splash-and-river pass a separate product only non-swimmers are offered?</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>The guest must actively agree on screen before capture. The notice-only option is not offered.</t>
+          <t>The answer filters products ('Help me choose'); the vest is an add-on; the splash-and-river pass is its own product.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Your data protection counsel</t>
+          <t>Your operations and safety team</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
@@ -1002,32 +1002,32 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Identity verification provider</t>
+          <t>Popular routes card</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Do you use an external identity-verification provider for guest ID documents, and if so which one?</t>
+          <t>The popular routes cards need a starting fare, a featured order and an image or badge per route. Should these be set per route in the back office?</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Money your customers pay or get back</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Guest ID documents are reviewed by your staff.</t>
+          <t>Routes carry a featured order and an image; the starting fare is computed from the lowest fare.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Your operations team</t>
+          <t>Your transport team</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -1038,32 +1038,32 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Tax documents</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Biometric retention by law</t>
+          <t>B2C e-invoices</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>What minimum or maximum retention does the law require for Face Pass, Face Tag and failed or abandoned captures, in each region you operate? (Asked before; restated with what we built.)</t>
+          <t>Are e-invoices to consumers (B2C) outside the first phase of the UAE mandate for you, so only B2B invoices go through the provider at launch? (ADR-0062)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Face Tag deleted once the ticket is fully used; Face Pass retention set by each venue. The legal limit you confirm becomes a floor no venue setting can go below.</t>
+          <t>B2B invoices go through the provider; B2C receipts are issued by the platform and can be switched to the provider per venue when your mandate covers them.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Your data protection counsel</t>
+          <t>Your finance team</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr"/>
@@ -1074,17 +1074,17 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Biometrics for children</t>
+          <t>What 99.99% covers</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Adults may have face data stored with their consent. For guests under 18, should face capture (Face Pass, Face Tag) be excluded entirely, or allowed with a consent form signed by a parent or guardian? (Raised in the 30 September meeting.)</t>
+          <t>Which services does the 99.99% availability commitment cover: the whole platform, or the guest purchase and admission path only? And do you accept a separate target per tier (for example 99.99% for purchase and admission, 99.9% for back office and reporting)? (ADR-0060)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Face capture is not offered to guests under 18 until you decide; with guardian consent, the guardian's signed consent is recorded against the child's ticket before capture.</t>
+          <t>Purchase and admission are designed to 99.99%; back office, reporting and AI to 99.9%.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Your data protection counsel</t>
+          <t>Your IT owner</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -1110,32 +1110,32 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Forecasting</t>
+          <t>Availability</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Weather data</t>
+          <t>Zone-redundant hosting cost</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Do you approve a commercial weather data service as an input to attendance forecasting, and its monthly cost?</t>
+          <t>99.99% needs zone-redundant hosting in UAE North: about USD 8,050 a month against about USD 4,530 without it. Do you accept that cost for production? (ADR-0060, the Azure cost sheet)</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>A cost you approve</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Forecasts run on sales history, bookings on hand and the calendar (holidays, Ramadan) without weather until you approve.</t>
+          <t>Production is costed zone-redundant; pre-production is not.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Your commercial team</t>
+          <t>Your budget owner</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
@@ -1146,32 +1146,32 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Design sign-off</t>
+          <t>Where face templates are stored</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Name one design reviewer who signs off each wireframe batch within 3 working days.</t>
+          <t>Where may face templates be stored: only inside the facial-reader vendor's system at the venue, or also in the platform in UAE North (encrypted, with a key per tenant)? (ADR-0063)</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>A name only you can give</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Front-end screens are accepted only after that sign-off (decided 28 September).</t>
+          <t>Templates stay with the reader vendor; the platform keeps only a reference and the guest's consent.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Your product owner</t>
+          <t>Your data protection officer</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
@@ -1182,32 +1182,32 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Payment sandboxes</t>
+          <t>Face capture on a notice</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Send Stripe and Network International sandbox credentials, and name the finance or payments owner, by a date we agree together.</t>
+          <t>May a guest be enrolled for Face Tag on a displayed notice alone, with no action from them, under the UAE PDPL?</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Accounts only you hold</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Checkout's declined, unknown and reconcile paths cannot be tested without a sandbox.</t>
+          <t>The guest must actively agree on screen before capture. The notice-only option is not offered.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Your finance / payments owner</t>
+          <t>Your data protection counsel</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr"/>
@@ -1218,32 +1218,32 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Cloud event broker</t>
+          <t>Identity verification provider</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Which broker should carry the platform's events in the cloud: RabbitMQ or Kafka? We need your answer before 12 October (the second week of the first sprint), so that the first purchase can be proven end to end by 23 October. Why it matters: every sale reaches ticketing, the ledger and stock through this broker, so it must keep each order's events in sequence, set aside messages that fail, and run in the UAE. Our recommendation is RabbitMQ, ideally as a managed service in the Azure UAE North region if one is available there: it fits this workload, it is simpler to run, and venues that run on their own premises use RabbitMQ anyway. Kafka is the better choice only if you want to replay the history of events from the broker itself.</t>
+          <t>Do you use an external identity-verification provider for guest ID documents, and if so which one?</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>A platform and running cost you choose</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Everything is built behind one interface and tested on RabbitMQ, so either answer works; only the cloud setup waits for your choice.</t>
+          <t>Guest ID documents are reviewed by your staff.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Your IT / infrastructure owner</t>
+          <t>Your operations team</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr"/>
@@ -1254,32 +1254,32 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>POS terminal</t>
+          <t>Biometric retention by law</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Which POS terminal will the cashiers use: make, model and operating system (Windows, Android or iPad)? Your hardware list names the receipt printer, cash drawer, customer display and scanner, but not the terminal.</t>
+          <t>What minimum or maximum retention does the law require for Face Pass, Face Tag and failed or abandoned captures, in each region you operate? (Asked before; restated with what we built.)</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>The POS is built as an app that works offline and drives the printer, drawer and display through standard drivers. We assume a Windows touch terminal (the HP cash drawer, display and scanner on your list suggest an HP POS system); the operating system decides how those devices are driven, so we need it before the first sprint ends.</t>
+          <t>Face Tag deleted once the ticket is fully used; Face Pass retention set by each venue. The legal limit you confirm becomes a floor no venue setting can go below.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your data protection counsel</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr"/>
@@ -1290,32 +1290,32 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Kitchen display</t>
+          <t>Biometrics for children</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Which kitchen display screens and kitchen printers will the kitchens use? Your hardware list says "decide later", and the kitchen display is in the first release.</t>
+          <t>Adults may have face data stored with their consent. For guests under 18, should face capture (Face Pass, Face Tag) be excluded entirely, or allowed with a consent form signed by a parent or guardian? (Raised in the 30 September meeting.)</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>The kitchen display is built as a browser screen that runs on any wall-mounted touch screen or tablet, with kitchen tickets also printable on an Epson-compatible printer.</t>
+          <t>Face capture is not offered to guests under 18 until you decide; with guardian consent, the guardian's signed consent is recorded against the child's ticket before capture.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Your F&amp;B / operations team</t>
+          <t>Your data protection counsel</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr"/>
@@ -1326,32 +1326,32 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Forecasting</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Card payment terminals</t>
+          <t>Weather data</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Which card payment terminals will the POS and the kiosks use, and from which provider (Stripe Terminal, Network International, or another)? They are not on your hardware list.</t>
+          <t>Do you approve a commercial weather data service as an input to attendance forecasting, and its monthly cost?</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>A device and a merchant contract only you hold</t>
+          <t>A cost you approve</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Card payments at the POS go through the payment provider's terminal, paired to one POS; the POS never sees a card number. Until you name the terminal, testing uses the provider's simulator.</t>
+          <t>Forecasts run on sales history, bookings on hand and the calendar (holidays, Ramadan) without weather until you approve.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Your finance / payments owner</t>
+          <t>Your commercial team</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr"/>
@@ -1362,32 +1362,32 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Accounts and people</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>NFC and RFID media</t>
+          <t>Design sign-off</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Which NFC readers (your list says "China", still open) and RFID readers (Kaptur, still open), and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
+          <t>Name one design reviewer who signs off each wireframe batch within 3 working days.</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>A name only you can give</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Wristbands and cards are read by their unique id and a secured application on the chip; nothing of value is stored on the chip itself. The exact chip type sets how the encoder is driven.</t>
+          <t>Front-end screens are accepted only after that sign-off (decided 28 September).</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your product owner</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr"/>
@@ -1398,32 +1398,32 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Accounts and people</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Staff and flying POS devices</t>
+          <t>Payment sandboxes</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Will the staff app and the flying (handheld) POS run on the Chainway C66 handhelds on your list, or on other phones or tablets?</t>
+          <t>Send Stripe and Network International sandbox credentials, and name the finance or payments owner, by a date we agree together.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>Accounts only you hold</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Both are built as one Android app for the Chainway C66, which also scans and prints over Bluetooth to the Zebra printer.</t>
+          <t>Checkout's declined, unknown and reconcile paths cannot be tested without a sandbox.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Your operations team</t>
+          <t>Your finance / payments owner</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr"/>
@@ -1434,32 +1434,32 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Devices in the requirements but not on your hardware list</t>
+          <t>Cloud event broker</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
+          <t>Which broker should carry the platform's events in the cloud: RabbitMQ or Kafka? We need your answer before 12 October (the second week of the first sprint), so that the first purchase can be proven end to end by 23 October. Why it matters: every sale reaches ticketing, the ledger and stock through this broker, so it must keep each order's events in sequence, set aside messages that fail, and run in the UAE. Our recommendation is RabbitMQ, ideally as a managed service in the Azure UAE North region if one is available there: it fits this workload, it is simpler to run, and venues that run on their own premises use RabbitMQ anyway. Kafka is the better choice only if you want to replay the history of events from the broker itself.</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>A device only you buy</t>
+          <t>A platform and running cost you choose</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
+          <t>Everything is built behind one interface and tested on RabbitMQ, so either answer works; only the cloud setup waits for your choice.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Your operations / IT team</t>
+          <t>Your IT / infrastructure owner</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr"/>
@@ -1470,32 +1470,32 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Messaging providers</t>
+          <t>POS terminal</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
+          <t>Which POS terminal will the cashiers use: make, model and operating system (Windows, Android or iPad)? Your hardware list names the receipt printer, cash drawer, customer display and scanner, but not the terminal.</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
+          <t>The POS is built as an app that works offline and drives the printer, drawer and display through standard drivers. We assume a Windows touch terminal (the HP cash drawer, display and scanner on your list suggest an HP POS system); the operating system decides how those devices are driven, so we need it before the first sprint ends.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr"/>
@@ -1506,32 +1506,32 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Accounting system</t>
+          <t>Kitchen display</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
+          <t>Which kitchen display screens and kitchen printers will the kitchens use? Your hardware list says "decide later", and the kitchen display is in the first release.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>A system and a format only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
+          <t>The kitchen display is built as a browser screen that runs on any wall-mounted touch screen or tablet, with kitchen tickets also printable on an Epson-compatible printer.</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Your finance team</t>
+          <t>Your F&amp;B / operations team</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr"/>
@@ -1542,32 +1542,32 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass</t>
+          <t>Card payment terminals</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
+          <t>Which card payment terminals will the POS and the kiosks use, and from which provider (Stripe Terminal, Network International, or another)? They are not on your hardware list.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device and a merchant contract only you hold</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
+          <t>Card payments at the POS go through the payment provider's terminal, paired to one POS; the POS never sees a card number. Until you name the terminal, testing uses the provider's simulator.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Your IT team</t>
+          <t>Your finance / payments owner</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr"/>
@@ -1578,32 +1578,32 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>App stores and digital wallets</t>
+          <t>NFC and RFID media</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
+          <t>Which NFC readers (your list says "China", still open) and RFID readers (Kaptur, still open), and which wristband and card chip type (for example MIFARE DESFire) will be used at gates and for cashless payments, and which device encodes the wristbands?</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
+          <t>Wristbands and cards are read by their unique id and a secured application on the chip; nothing of value is stored on the chip itself. The exact chip type sets how the encoder is driven.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr"/>
@@ -1614,32 +1614,32 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Tourism authority reporting</t>
+          <t>Staff and flying POS devices</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
+          <t>Will the staff app and the flying (handheld) POS run on the Chainway C66 handhelds on your list, or on other phones or tablets?</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
+          <t>Both are built as one Android app for the Chainway C66, which also scans and prints over Bluetooth to the Zebra printer.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Your compliance / finance team</t>
+          <t>Your operations team</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr"/>
@@ -1650,32 +1650,32 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Named third-party services</t>
+          <t>Devices in the requirements but not on your hardware list</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
+          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Your commercial / operations team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr"/>
@@ -1686,32 +1686,32 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Venue data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>3D venue model for in-park navigation</t>
+          <t>Messaging providers</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>In-park 3D navigation is built into the guest app, as agreed on 30 September, and needs two files for each venue: a 3D model of the venue (a GLB file) and a pathway and location file (the walkable paths, and where each ride, outlet, shop and facility is, linked to its catalogue item), with two or more surveyed GPS points so the model lines up with the guest's position. Will you supply these for each venue, or commission a 3D vendor to produce them, and by when? We will send the file specification.</t>
+          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Your venue's own asset, or a cost you approve</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>In-park navigation runs on the 2D park map, with the same routes and live GPS, until a venue's model is supplied; the 3D view switches on per venue when its files pass the platform's checks.</t>
+          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Your operations / venue team</t>
+          <t>Your IT / marketing team</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -1722,30 +1722,34 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Guardian consent for a minor's Face Pass (sent before)</t>
+          <t>Accounting system</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
+          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A system and a format only you hold</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr"/>
+          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Your finance team</t>
+        </is>
+      </c>
       <c r="H30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1754,30 +1758,34 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>The age of a minor (sent before)</t>
+          <t>UAE Pass</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Below what age is a guest a minor?</t>
+          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr"/>
+          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Your IT team</t>
+        </is>
+      </c>
       <c r="H31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1786,30 +1794,34 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Guest document retention (sent before)</t>
+          <t>App stores and digital wallets</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>How long is each kind of guest document kept?</t>
+          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr"/>
+          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Your IT / marketing team</t>
+        </is>
+      </c>
       <c r="H32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
@@ -1818,30 +1830,34 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Refunds</t>
+          <t>Government</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Cancelled event after a resale (sent before)</t>
+          <t>Tourism authority reporting</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
+          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Money your customers pay or get back</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr"/>
+          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Your compliance / finance team</t>
+        </is>
+      </c>
       <c r="H33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
@@ -1855,12 +1871,12 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Facial-reader vendor (sent before)</t>
+          <t>Named third-party services</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1870,10 +1886,14 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr"/>
+          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Your commercial / operations team</t>
+        </is>
+      </c>
       <c r="H34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1882,30 +1902,34 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Venue data</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Approved libraries (sent before)</t>
+          <t>3D venue model for in-park navigation</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+          <t>In-park 3D navigation is built into the guest app, as agreed on 30 September, and needs two files for each venue: a 3D model of the venue (a GLB file) and a pathway and location file (the walkable paths, and where each ride, outlet, shop and facility is, linked to its catalogue item), with two or more surveyed GPS points so the model lines up with the guest's position. Will you supply these for each venue, or commission a 3D vendor to produce them, and by when? We will send the file specification.</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Your venue's own asset, or a cost you approve</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr"/>
+          <t>In-park navigation runs on the 2D park map, with the same routes and live GPS, until a venue's model is supplied; the 3D view switches on per venue when its files pass the platform's checks.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Your operations / venue team</t>
+        </is>
+      </c>
       <c r="H35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1914,17 +1938,17 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Price tests on live customers (sent before)</t>
+          <t>Guardian consent for a minor's Face Pass (sent before)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -1934,7 +1958,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr"/>
@@ -1946,17 +1970,17 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Cooling-off after auto-renewal (sent before)</t>
+          <t>The age of a minor (sent before)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+          <t>Below what age is a guest a minor?</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -1966,14 +1990,206 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="7" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Guest data</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Guest document retention (sent before)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>How long is each kind of guest document kept?</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
+      <c r="H38" s="7" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Refunds</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Cancelled event after a resale (sent before)</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Money your customers pay or get back</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="7" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Suppliers</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Facial-reader vendor (sent before)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>A name, account or vendor only you hold</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Accounts and people</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Approved libraries (sent before)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>A name, account or vendor only you hold</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr"/>
+      <c r="H41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Price tests on live customers (sent before)</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr"/>
+      <c r="H42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Cooling-off after auto-renewal (sent before)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr"/>
+      <c r="H43" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
TICVAI: Decisions Register and ADR-0060 carry the re-priced cost ($8,050 with HA, $5,550 without) and ADR-0060's four availability tiers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Decisions Register.xlsx
+++ b/ticvai/handoff/TICVAI - Decisions Register.xlsx
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Which services does the 99.99% availability commitment cover: the whole platform, or the guest purchase and admission path only? And do you accept a separate target per tier (for example 99.99% for purchase and admission, 99.9% for back office and reporting)? (ADR-0060)</t>
+          <t>Which services does the 99.99% availability commitment cover: the whole platform, or the guest purchase and admission path only? And do you accept a separate target per tier: 99.99% at the venue (gates, POS, kitchen display, which keep working offline), 99.95% for online sales, 99.9% for the back office and reporting, 99.5% for AI? (ADR-0060)</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Purchase and admission are designed to 99.99%; back office, reporting and AI to 99.9%.</t>
+          <t>Built to those four tiers: the venue at 99.99% because it runs offline, online sales at 99.95%, back office 99.9%, AI 99.5%.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>99.99% needs zone-redundant hosting in UAE North: about USD 8,050 a month against about USD 4,530 without it. Do you accept that cost for production? (ADR-0060, the Azure cost sheet)</t>
+          <t>The availability targets need high-availability hosting in UAE North: about USD 8,050 a month for a production cell, against about USD 5,550 without it (re-priced 1 October). Do you accept that cost for production? (ADR-0060, the Azure cost sheet)</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -28935,12 +28935,12 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>identity: createAccessPolicy</t>
+          <t>identity: createAuthorisationPolicy</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity now has attribute-based policies: createAccessPolicy writes an AccessPolicy of AccessCondition rows (attribute, operator, value) with an effect, evaluated by evaluateAccess against an AccessContext. access also carries its own dynamic policy set (setVisualDynamicPolicy, AccessDynamicPolicy) - two policy models to reconcile.</t>
+          <t>re-traced 29 September: identity now has attribute-based policies: createAuthorisationPolicy writes an AuthorisationPolicy of AccessCondition rows (attribute, operator, value) with an effect, evaluated by evaluateAccess against an AccessContext. access also carries its own dynamic policy set (setVisualDynamicPolicy, AccessDynamicPolicy) - two policy models to reconcile.</t>
         </is>
       </c>
     </row>
@@ -28972,7 +28972,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has location.scopePath and venue.id; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has location.scopePath and venue.id; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29004,7 +29004,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has time.ofDay, time.withinOperatingHours and employee.onShift; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). AccessPolicy.effectiveFrom/effectiveTo add a validity window. ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has time.ofDay, time.withinOperatingHours and employee.onShift; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). AuthorisationPolicy.effectiveFrom/effectiveTo add a validity window. ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29036,7 +29036,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has ticket.status and event.status; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has ticket.status and event.status; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29063,12 +29063,12 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>identity: createAccessPolicy</t>
+          <t>identity: createAuthorisationPolicy</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: createAccessPolicy ('write a policy without writing code') takes conditions from a fixed AccessCondition vocabulary with allMustMatch/anyMayMatch combining; updateAccessPolicy edits as a new version. access setVisualDynamicPolicy is the no-code builder screen.</t>
+          <t>re-traced 29 September: createAuthorisationPolicy ('write a policy without writing code') takes conditions from a fixed AccessCondition vocabulary with allMustMatch/anyMayMatch combining; updateAuthorisationPolicy edits as a new version. access setVisualDynamicPolicy is the no-code builder screen.</t>
         </is>
       </c>
     </row>
@@ -29132,7 +29132,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has user.attribute (key names the attribute); policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has user.attribute (key names the attribute); policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29164,7 +29164,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has employee.attribute and employee.onShift; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has employee.attribute and employee.onShift; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29196,7 +29196,7 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has membership.tier and membership.status; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has membership.tier and membership.status; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29228,7 +29228,7 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has accreditation.type and accreditation.status; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has accreditation.type and accreditation.status; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29260,7 +29260,7 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has customer.segment; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has customer.segment; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29292,7 +29292,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has resource.classification; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has resource.classification; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29324,7 +29324,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has venue.attribute and venue.id; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has venue.attribute and venue.id; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29356,7 +29356,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has attraction.attribute; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). AccessContext.attractionId supplies the attraction. ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has attraction.attribute; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). AccessContext.attractionId supplies the attraction. ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29388,7 +29388,7 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has device.kind, device.id and device.trusted; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). AccessContext.deviceId supplies the device. ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has device.kind, device.id and device.trusted; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). AccessContext.deviceId supplies the device. ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29420,7 +29420,7 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has time.dayOfWeek; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has time.dayOfWeek; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29452,7 +29452,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has time.season; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has time.season; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29484,7 +29484,7 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has event.id and event.status; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). AccessContext.eventId supplies the event. ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has event.id and event.status; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). AccessContext.eventId supplies the event. ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29516,7 +29516,7 @@
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has capacity.utilisationPercent; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has capacity.utilisationPercent; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29548,7 +29548,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has occupancy.level; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has occupancy.level; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29580,7 +29580,7 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity AccessCondition.attribute has risk.score; policies are written with createAccessPolicy and decided by evaluateAccess (AccessContext carries the inputs). The score's bands are configured by access setRiskScoringConfig. ABAC now exists in identity, so the BL-110 gap is closed.</t>
+          <t>re-traced 29 September: identity AccessCondition.attribute has risk.score; policies are written with createAuthorisationPolicy and decided by evaluateAccess (AccessContext carries the inputs). The score's bands are configured by access setRiskScoringConfig. ABAC now exists in identity, so the BL-110 gap is closed.</t>
         </is>
       </c>
     </row>
@@ -29612,7 +29612,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: access setVisualDynamicPolicy is the Visual Dynamic Policy Builder (IF/AND/OR/NOT/IN, pack p.136) writing conditionExpression, result and priority, with the attribute catalogue (listAccessAttributeCatalog) and simulation (simulatePolicyConflictImpact). It writes access AccessDynamicPolicy, not identity AccessPolicy.</t>
+          <t>re-traced 29 September: access setVisualDynamicPolicy is the Visual Dynamic Policy Builder (IF/AND/OR/NOT/IN, pack p.136) writing conditionExpression, result and priority, with the attribute catalogue (listAccessAttributeCatalog) and simulation (simulatePolicyConflictImpact). It writes access AccessDynamicPolicy, not identity AuthorisationPolicy.</t>
         </is>
       </c>
     </row>
@@ -29639,12 +29639,12 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>identity: listAccessPolicyTemplates</t>
+          <t>identity: listAuthorisationPolicyTemplates</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity listAccessPolicyTemplates returns reusable policy shapes; a template is an AccessPolicy with isTemplate true, written through createAccessPolicy.</t>
+          <t>re-traced 29 September: identity listAuthorisationPolicyTemplates returns reusable policy shapes; a template is an AuthorisationPolicy with isTemplate true, written through createAuthorisationPolicy.</t>
         </is>
       </c>
     </row>
@@ -29671,12 +29671,12 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>identity: updateAccessPolicy</t>
+          <t>identity: updateAuthorisationPolicy</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: every identity updateAccessPolicy writes a new AccessPolicy.version; getAccessPolicy reads one at a version and listAccessPolicyHistory lists them (AccessPolicyVersion). access also has rollbackAccessPolicy for its dynamic policies.</t>
+          <t>re-traced 29 September: every identity updateAuthorisationPolicy writes a new AuthorisationPolicy.version; getAuthorisationPolicy reads one at a version and listAuthorisationPolicyHistory lists them (AuthorisationPolicyVersion). access also has rollbackAccessPolicy for its dynamic policies.</t>
         </is>
       </c>
     </row>
@@ -29703,12 +29703,12 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>identity: simulateAccessPolicy</t>
+          <t>identity: simulateAuthorisationPolicy</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity simulateAccessPolicy decides a draft policy against an AccessContext before it is active (same shape as evaluateAccess); access simulatePolicyConflictImpact does the same for dynamic policies.</t>
+          <t>re-traced 29 September: identity simulateAuthorisationPolicy decides a draft policy against an AccessContext before it is active (same shape as evaluateAccess); access simulatePolicyConflictImpact does the same for dynamic policies.</t>
         </is>
       </c>
     </row>
@@ -29735,12 +29735,12 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>identity: setAccessPolicyState</t>
+          <t>identity: setAuthorisationPolicyState</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity setAccessPolicyState moves a policy draft -&gt; pendingApproval -&gt; active (submit, approve, activate, retire); status cannot be set by create/update, so approval cannot be skipped; AccessPolicyVersion.approvedBy records the approver.</t>
+          <t>re-traced 29 September: identity setAuthorisationPolicyState moves a policy draft -&gt; pendingApproval -&gt; active (submit, approve, activate, retire); status cannot be set by create/update, so approval cannot be skipped; AuthorisationPolicyVersion.approvedBy records the approver.</t>
         </is>
       </c>
     </row>
@@ -29772,7 +29772,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity evaluateAccess is the single central decision point (AccessDecision.decidedBy central), with getAccessPolicyBundle for device-side evaluation offline.</t>
+          <t>re-traced 29 September: identity evaluateAccess is the single central decision point (AccessDecision.decidedBy central), with getAuthorisationPolicyBundle for device-side evaluation offline.</t>
         </is>
       </c>
     </row>
@@ -29799,12 +29799,12 @@
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>identity: AccessPolicy</t>
+          <t>identity: AuthorisationPolicy</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: AccessPolicy.delegatedAdminRoleIds names roles that may edit the policy without being platform administrators, set through createAccessPolicy/updateAccessPolicy.</t>
+          <t>re-traced 29 September: AuthorisationPolicy.delegatedAdminRoleIds names roles that may edit the policy without being platform administrators, set through createAuthorisationPolicy/updateAuthorisationPolicy.</t>
         </is>
       </c>
     </row>
@@ -29863,12 +29863,12 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>identity: listAccessPolicyHistory</t>
+          <t>identity: listAuthorisationPolicyHistory</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: identity listAccessPolicyHistory returns every version with changedBy, changedAt, reason, approvedBy and the previous and current policy.</t>
+          <t>re-traced 29 September: identity listAuthorisationPolicyHistory returns every version with changedBy, changedAt, reason, approvedBy and the previous and current policy.</t>
         </is>
       </c>
     </row>
@@ -29895,12 +29895,12 @@
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>identity: AccessPolicy</t>
+          <t>identity: AuthorisationPolicy</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: AccessPolicy.scopePath scopes a policy to a tenant (or below); tenant, venue and cross-venue policies are one mechanism by scope-path prefix.</t>
+          <t>re-traced 29 September: AuthorisationPolicy.scopePath scopes a policy to a tenant (or below); tenant, venue and cross-venue policies are one mechanism by scope-path prefix.</t>
         </is>
       </c>
     </row>
@@ -29927,12 +29927,12 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>identity: AccessPolicy</t>
+          <t>identity: AuthorisationPolicy</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: AccessPolicy.scopePath at a node above several venues (e.g. uae.dubai) applies to every venue beneath it by prefix inheritance; AccessCondition venue.id with operator in narrows to a chosen set.</t>
+          <t>re-traced 29 September: AuthorisationPolicy.scopePath at a node above several venues (e.g. uae.dubai) applies to every venue beneath it by prefix inheritance; AccessCondition venue.id with operator in narrows to a chosen set.</t>
         </is>
       </c>
     </row>
@@ -30092,7 +30092,7 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September (build): per-policy effectiveness over a period for gate policies (listDynamicPolicyEffectiveness: triggers, allow/deny/review/step-up, supervisor overrides, override rate, never-triggered, daily trend; ScanEvent now records the deciding dynamicPolicyId/version/result) and for software-permission policies (identity listAccessPolicyEffectiveness).</t>
+          <t>re-traced 29 September (build): per-policy effectiveness over a period for gate policies (listDynamicPolicyEffectiveness: triggers, allow/deny/review/step-up, supervisor overrides, override rate, never-triggered, daily trend; ScanEvent now records the deciding dynamicPolicyId/version/result) and for software-permission policies (identity listAuthorisationPolicyEffectiveness).</t>
         </is>
       </c>
     </row>
@@ -31852,7 +31852,7 @@
       </c>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: attribute-based policies narrow or extend role grants: AccessPolicy.conditions on user, resource, environment and time, and evaluateAccess decides per request and says which condition failed. BL-110 is built in identity</t>
+          <t>re-traced 29 September: attribute-based policies narrow or extend role grants: AuthorisationPolicy.conditions on user, resource, environment and time, and evaluateAccess decides per request and says which condition failed. BL-110 is built in identity</t>
         </is>
       </c>
     </row>
@@ -31911,12 +31911,12 @@
       </c>
       <c r="E155" s="3" t="inlineStr">
         <is>
-          <t>identity: createAccessPolicy</t>
+          <t>identity: createAuthorisationPolicy</t>
         </is>
       </c>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: policies are data written without code (createAccessPolicy): conditions with combining logic, approval through setAccessPolicyState routed to approvals, and reusable templates. The visual builder is the screen over this operation</t>
+          <t>re-traced 29 September: policies are data written without code (createAuthorisationPolicy): conditions with combining logic, approval through setAuthorisationPolicyState routed to approvals, and reusable templates. The visual builder is the screen over this operation</t>
         </is>
       </c>
     </row>
@@ -31943,12 +31943,12 @@
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>identity: listAccessPolicyTemplates</t>
+          <t>identity: listAuthorisationPolicyTemplates</t>
         </is>
       </c>
       <c r="F156" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September: reusable policy templates (listAccessPolicyTemplates, AccessPolicy.isTemplate), applied at any scope node (scopePath covers department, business unit, venue, attraction) and to roles. A sales channel is expressed as a condition</t>
+          <t>re-traced 29 September: reusable policy templates (listAuthorisationPolicyTemplates, AuthorisationPolicy.isTemplate), applied at any scope node (scopePath covers department, business unit, venue, attraction) and to roles. A sales channel is expressed as a condition</t>
         </is>
       </c>
     </row>
@@ -31975,12 +31975,12 @@
       </c>
       <c r="E157" s="3" t="inlineStr">
         <is>
-          <t>identity: restoreAccessPolicyVersion</t>
+          <t>identity: restoreAuthorisationPolicyVersion</t>
         </is>
       </c>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September (build): versions kept with who and why (listAccessPolicyHistory, previous/current for comparison, getAccessPolicy by version) and rollback to a previously approved version through restoreAccessPolicyVersion (new pendingApproval version, never a rewind; 409 for a never-approved target).</t>
+          <t>re-traced 29 September (build): versions kept with who and why (listAuthorisationPolicyHistory, previous/current for comparison, getAuthorisationPolicy by version) and rollback to a previously approved version through restoreAuthorisationPolicyVersion (new pendingApproval version, never a rewind; 409 for a never-approved target).</t>
         </is>
       </c>
     </row>
@@ -32012,7 +32012,7 @@
       </c>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September (build): sandbox testing of draft policies (simulateAccessPolicy, resolvePermissions) plus listPermissionFindings for excessive (unused in lookback), missing (repeatedly denied, held by role peers) and conflicting (segregation) permissions, optionally as if a draft policy were active (draftPolicyId).</t>
+          <t>re-traced 29 September (build): sandbox testing of draft policies (simulateAuthorisationPolicy, resolvePermissions) plus listPermissionFindings for excessive (unused in lookback), missing (repeatedly denied, held by role peers) and conflicting (segregation) permissions, optionally as if a draft policy were active (draftPolicyId).</t>
         </is>
       </c>
     </row>
@@ -32044,7 +32044,7 @@
       </c>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>re-traced 29 September (AI build): getEntityRisk scores staff, account, device and credential entities from composite signals (login events with hashed device, velocity, history); rules-first producer until a model is promoted per tenant. Missing: permission sensitivity as a signal and a risk-driven step-up; identity AccessPolicy can test risk.score but only permits or denies, and step-up is only on device/location restriction (setPasswordPolicy onViolation requireStepUp).</t>
+          <t>re-traced 29 September (AI build): getEntityRisk scores staff, account, device and credential entities from composite signals (login events with hashed device, velocity, history); rules-first producer until a model is promoted per tenant. Missing: permission sensitivity as a signal and a risk-driven step-up; identity AuthorisationPolicy can test risk.score but only permits or denies, and step-up is only on device/location restriction (setPasswordPolicy onViolation requireStepUp).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TICVAI r4: the hardware workbook (Boca settled, client documents and next step columns) and the Decisions Register (six BOCA questions, pending, not sent) rebuilt by their hand-run generators (CHG-R4-002)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI - Decisions Register.xlsx
+++ b/ticvai/handoff/TICVAI - Decisions Register.xlsx
@@ -17,12 +17,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements closed" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'For you to answer'!$A$1:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Audit decisions'!$A$1:$G$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rev 3 prototype feedback'!$A$1:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Agreed operations'!$A$1:$E$575</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Operations added'!$A$1:$D$207</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'AI decisions'!$A$1:$C$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'AI decisions'!$A$1:$C$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Requirements closed'!$A$1:$F$531</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Prepared by Softlabs · 1 October 2026 · generated from the specification package</t>
+          <t>Prepared by Softlabs · 5 October 2026 · generated from the specification package</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1655,12 +1655,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Devices in the requirements but not on your hardware list</t>
+          <t>BOCA printer: model and count (pending, not sent)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
+          <t>Which BOCA model or models will you use (Lemur, Lemur-C or another), and how many at each kiosk, POS and box office?</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
+          <t>Tickets and wristbands print in BOCA's FGL command language, which the BOCA models share; we build and test against an emulated printer until the unit arrives.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -1686,32 +1686,32 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Messaging providers</t>
+          <t>BOCA printer: connection and host (pending, not sent)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
+          <t>How will each BOCA printer connect (USB, Ethernet or serial), and which operating system runs the kiosks and POS it is attached to? That decides whether we print through the Windows driver or send FGL directly over the network from our device app.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
+          <t>We send FGL directly to the printer (over the network or USB) from the device app, so no operating-system driver is needed; the Windows driver is the fallback.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr"/>
@@ -1722,32 +1722,32 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Accounting system</t>
+          <t>BOCA printer: ticket and wristband stock (pending, not sent)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
+          <t>Which ticket and wristband stock will you use: sizes, thermal or other, pre-printed backgrounds, and the black-mark and cut settings?</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>A system and a format only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
+          <t>Ticket and wristband layouts come from the ticket designer at a standard ticket and wristband size; the stock settings are per printer.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Your finance team</t>
+          <t>Your operations team</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr"/>
@@ -1758,32 +1758,32 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass</t>
+          <t>BOCA printer: RFID encoding (pending, not sent)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
+          <t>Are RFID-encoded wristbands or tickets in scope? If so, which chip, what data is written (the credential id only?), and do the gates' readers read it?</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
+          <t>RFID encoding on the BOCA Lemur is built behind a switch, off, until you confirm; tickets and wristbands carry the printed QR code.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Your IT team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr"/>
@@ -1794,32 +1794,32 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>App stores and digital wallets</t>
+          <t>BOCA printer: arrival and contact (pending, not sent)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
+          <t>When will the printer reach our India office, and who is the BOCA technical contact for questions?</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>An account only you hold</t>
+          <t>A name, account or vendor only you hold</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
+          <t>The driver is built and tested on an emulated printer now; the test on the real printer is scheduled when it arrives.</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Your IT / marketing team</t>
+          <t>Muhamed Allam</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr"/>
@@ -1830,32 +1830,32 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Tourism authority reporting</t>
+          <t>BOCA printer: mandated settings (pending, not sent)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
+          <t>Does the venue mandate any printer firmware version or printer settings we must keep?</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
+          <t>We keep BOCA's factory settings and change only what printing needs (the stock, the cut).</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Your compliance / finance team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr"/>
@@ -1866,32 +1866,32 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Named third-party services</t>
+          <t>Devices in the requirements but not on your hardware list</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
+          <t>Your requirements include parking cameras and barriers, queue and occupancy sensors and beacons, game readers and redemption terminals, electronic lockers and digital signage, but your hardware list names none of them. Which are in scope, and which make and model for each?</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>A device only you buy</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+          <t>Each is built behind a standard device interface and connected when you name the device; until then they are out of the first release.</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Your commercial / operations team</t>
+          <t>Your operations / IT team</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr"/>
@@ -1902,32 +1902,32 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Venue data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>3D venue model for in-park navigation</t>
+          <t>Messaging providers</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>In-park 3D navigation is built into the guest app, as agreed on 30 September, and needs two files for each venue: a 3D model of the venue (a GLB file) and a pathway and location file (the walkable paths, and where each ride, outlet, shop and facility is, linked to its catalogue item), with two or more surveyed GPS points so the model lines up with the guest's position. Will you supply these for each venue, or commission a 3D vendor to produce them, and by when? We will send the file specification.</t>
+          <t>Which SMS gateway and which email sending service will deliver tickets, codes and receipts, and will you use WhatsApp Business (whose account)?</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Your venue's own asset, or a cost you approve</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>In-park navigation runs on the 2D park map, with the same routes and live GPS, until a venue's model is supplied; the 3D view switches on per venue when its files pass the platform's checks.</t>
+          <t>Tickets and one-time codes are sent through a provider adapter; development uses a test mailbox and a test SMS sender. The first release needs the real SMS and email senders for guests to receive their tickets.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Your operations / venue team</t>
+          <t>Your IT / marketing team</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr"/>
@@ -1938,30 +1938,34 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Guardian consent for a minor's Face Pass (sent before)</t>
+          <t>Accounting system</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
+          <t>Which accounting or ERP system receives the platform's financial postings (for example SAP or Oracle), and in what format?</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>A system and a format only you hold</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr"/>
+          <t>The ledger exports its journal as a file per day in a documented format; an adapter for your system is built once you name it.</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Your finance team</t>
+        </is>
+      </c>
       <c r="H36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1970,30 +1974,34 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>The age of a minor (sent before)</t>
+          <t>UAE Pass</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Below what age is a guest a minor?</t>
+          <t>Is your organisation registered as a UAE Pass service provider, and who holds the credentials? Guests sign in with UAE Pass as well as a one-time code and social sign-in.</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr"/>
+          <t>UAE Pass sign-in is built against its staging environment and switched on when your credentials arrive; the other sign-in methods work without it.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Your IT team</t>
+        </is>
+      </c>
       <c r="H37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
@@ -2002,30 +2010,34 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Guest data</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Guest document retention (sent before)</t>
+          <t>App stores and digital wallets</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>How long is each kind of guest document kept?</t>
+          <t>Which Apple and Google developer accounts will publish each venue's app, and who holds the Apple Wallet and Google Wallet pass certificates?</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Law, a regulator or a third-party contract</t>
+          <t>An account only you hold</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr"/>
+          <t>Apps are built and signed in our test accounts; publishing and wallet passes wait for yours.</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Your IT / marketing team</t>
+        </is>
+      </c>
       <c r="H38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
@@ -2034,30 +2046,34 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Refunds</t>
+          <t>Government</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Cancelled event after a resale (sent before)</t>
+          <t>Tourism authority reporting</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
+          <t>Must the platform report visitor or sales figures to the Department of Economy and Tourism (Dubai) or the Department of Culture and Tourism (Abu Dhabi), and if so which reports and with which credentials?</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Money your customers pay or get back</t>
+          <t>Law, a regulator or a third-party contract</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr"/>
+          <t>No reporting to a tourism authority is built; the figures such a report needs are all in the reporting layer, so a report can be added once the rules are known.</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Your compliance / finance team</t>
+        </is>
+      </c>
       <c r="H39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2071,12 +2087,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Facial-reader vendor (sent before)</t>
+          <t>Named third-party services</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+          <t>Your requirements name dynamic pricing (Digonex), city passes (Go City), locker systems (Gantner, Metra) and third-party queue systems. Which of these do you use or plan to use?</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -2086,10 +2102,14 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr"/>
+          <t>Pricing rules, passes, lockers and queues are built into the platform; an outside service is connected through an adapter once you confirm it.</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Your commercial / operations team</t>
+        </is>
+      </c>
       <c r="H40" s="7" t="inlineStr"/>
     </row>
     <row r="41">
@@ -2098,30 +2118,34 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Accounts and people</t>
+          <t>Venue data</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Approved libraries (sent before)</t>
+          <t>3D venue model for in-park navigation</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+          <t>In-park 3D navigation is built into the guest app, as agreed on 30 September, and needs two files for each venue: a 3D model of the venue (a GLB file) and a pathway and location file (the walkable paths, and where each ride, outlet, shop and facility is, linked to its catalogue item), with two or more surveyed GPS points so the model lines up with the guest's position. Will you supply these for each venue, or commission a 3D vendor to produce them, and by when? We will send the file specification.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>A name, account or vendor only you hold</t>
+          <t>Your venue's own asset, or a cost you approve</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr"/>
+          <t>In-park navigation runs on the 2D park map, with the same routes and live GPS, until a venue's model is supplied; the 3D view switches on per venue when its files pass the platform's checks.</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Your operations / venue team</t>
+        </is>
+      </c>
       <c r="H41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2130,17 +2154,17 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Price tests on live customers (sent before)</t>
+          <t>Guardian consent for a minor's Face Pass (sent before)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+          <t>At what age must a guardian consent to a minor's Face Pass enrolment, in each jurisdiction?</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -2150,7 +2174,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>The signed-in adult enrols a linked child and is recorded as guardian. Counsel sets the age.</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr"/>
@@ -2162,17 +2186,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Consumer law</t>
+          <t>Guest data</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Cooling-off after auto-renewal (sent before)</t>
+          <t>The age of a minor (sent before)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+          <t>Below what age is a guest a minor?</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2182,14 +2206,206 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Kept open in the specification; the rest is built.</t>
+          <t>A guest with no date of birth is treated as a minor; the age is the one your counsel gives.</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="7" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Guest data</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Guest document retention (sent before)</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>How long is each kind of guest document kept?</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Kept until the purpose ends, then for the period your counsel sets.</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Refunds</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Cancelled event after a resale (sent before)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>When an event is cancelled after a ticket was resold, who is refunded and how much: the resale buyer at the resale price, the original buyer, or both? Is the seller's payout taken back?</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Money your customers pay or get back</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="7" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Suppliers</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Facial-reader vendor (sent before)</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Which facial-reader vendor have you contracted? It sets the SDK and the template format.</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>A name, account or vendor only you hold</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>The platform uses the SDK of the vendor you name; nothing vendor-specific is built before that.</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="7" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Accounts and people</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Approved libraries (sent before)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Who on your side approves the list of third-party libraries each part of the platform may use, and any addition to it?</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>A name, account or vendor only you hold</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>We draft the list from what the starters already ship (Serilog, OpenTelemetry to OTLP, health checks) and you approve it. Anything else needs one named approver on your side.</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="7" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Price tests on live customers (sent before)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Are A/B price tests on live customers allowed, and with what notice? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="7" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Consumer law</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Cooling-off after auto-renewal (sent before)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>What cooling-off rights apply after an auto-renewal charge? Not blocking: built as a venue setting that a person approves.</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Law, a regulator or a third-party contract</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Kept open in the specification; the rest is built.</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr"/>
+      <c r="H49" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H43"/>
+  <autoFilter ref="A1:H49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26572,7 +26788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -26627,7 +26843,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Managed Azure OpenAI re-billed per token; billing per selected module; 3 packages plus custom; module prices configured by TICVAI on the platform</t>
+          <t>Per-tenant AI residency class (ADR-0009, amended 2 October). UAE-only, the default and mandatory for government, bank and health tenants: Small = Core42 Compass GPT-4.1 mini (or GPT-4.1 Arabic 'Seraj' if it wins the Arabic golden set), Strong = Compass GPT-5, fallback OpenAI UAE (the in-cell gpt-oss-120b fallback was dropped on 3 October: we host no model unless a client asks, and the guard is the provider's content-safety service; CHG-R1S-002); Compass is reached through AiProviderKind openaiCompatible and billed through Azure Marketplace. Global allowed (a private venue opts in under PDPL Art. 23 with a vendor contract, DPIA and notice): Azure gpt-5-mini / gpt-6-sol Global Standard or the tenant's BYOK provider, fallback the UAE-only chain. On-premise: Qwen3.5 or gpt-oss; Strong Qwen3.5-122B, Falcon-H1 Arabic or Jais 2. Scale step: the UAE-only Small tier moves to Azure UAE North PTU (spillover off) when steady traffic nears about 100,000 calls a day. Billing stays per token, per selected module (3 packages plus custom; module prices configured by TICVAI). Vendor terms in writing before signing (DEC-541, open).</t>
         </is>
       </c>
     </row>
@@ -26644,7 +26860,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>UAE North for now; other regions configured tenant by tenant</t>
+          <t>In-UAE inference by default: every tenant is UAE-only unless it opts in to Global allowed (AI-D02); other regions are configured tenant by tenant.</t>
         </is>
       </c>
     </row>
@@ -26899,7 +27115,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Our proposal, adopted: each model carries a task-fitness band per agent task (AiModel.taskFitness: score, floor, ceiling, evaluation run); setAiProvider returns fitness warnings (underpowered, overpowered, unscored) and never blocks the choice</t>
+          <t>Amended: each model still carries a task-fitness band per agent task (AiModel.taskFitness: score, floor, ceiling, evaluation run), and TICVAI curates the model per task; setAiProvider / setAiModel refuse a model outside the curated map for that task. A client cannot change the model per agent (cheaper models would break the AI functions).</t>
         </is>
       </c>
     </row>
@@ -26933,12 +27149,29 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>DEFERRED, not decided: to the dedicated AI workshop (client meeting 30 September, MoM 4.1; Allam). Position stated on the call, for the workshop to confirm: the AI agents behave the same whichever model a client selects, with only minor performance variation; we propose a recommended model per function; any extra cost of a provider or model the client chooses (for example ChatGPT) is borne by the client. Until the workshop, AI-D02 (managed Azure OpenAI, re-billed per token) stands as the default</t>
+          <t>Closed: with BYOK the AI engine maps each AI task to the client provider's equivalent model from TICVAI's curated range (tiers, not model names; docs/active/research/ai-ml-model-selection-2-october.md section 2.3), and usage is billed to the client's own key. Any BYOK provider other than OpenAI's UAE region is a cross-border transfer, so BYOK fits the Global-allowed residency class only (ADR-0009 section 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>AI-D21</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Which models may run each AI and ML task</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>TICVAI curates a range per AI and ML task: the best-suited model plus 3-4 alternatives where they exist (generative tiers Small, Strong, Reasoning; embeddings, reranking, moderation, PII detection, OCR and speech are platform-owned and never BYOK; every money path stays classical ML). The range is recorded in the AI design and seeded in the AI model catalogue; the individual picks are the research's recommendations (docs/active/research/ai-ml-model-selection-2-october.md sections 1 and 3) until the golden sets confirm them.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:C22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>